<commit_message>
feat: generate ebay search urls
</commit_message>
<xml_diff>
--- a/data/results.xlsx
+++ b/data/results.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.ebay.de/</t>
+          <t>https://www.ebay.de/sch/i.html?_nkw=532406713</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.ebay.de/</t>
+          <t>https://www.ebay.de/sch/i.html?_nkw=BPR6ES</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.ebay.de/</t>
+          <t>https://www.ebay.de/sch/i.html?_nkw=532187256</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.ebay.de/</t>
+          <t>https://www.ebay.de/sch/i.html?_nkw=GX160-AF</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.ebay.de/</t>
+          <t>https://www.ebay.de/sch/i.html?_nkw=P-0010038-X1HO0007</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: extend competitor product data
</commit_message>
<xml_diff>
--- a/data/results.xlsx
+++ b/data/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,10 +449,20 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Versand</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Verkaufte MengeBewertung</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Verkäufer</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -483,14 +493,20 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="G2" t="inlineStr">
+        <v>4.99</v>
+      </c>
+      <c r="G2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>ExampleSeller</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>https://www.ebay.de/sch/i.html?_nkw=532406713</t>
         </is>
@@ -521,14 +537,20 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="G3" t="inlineStr">
+        <v>4.99</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>ExampleSeller</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>https://www.ebay.de/sch/i.html?_nkw=BPR6ES</t>
         </is>
@@ -559,14 +581,20 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="G4" t="inlineStr">
+        <v>4.99</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>ExampleSeller</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>https://www.ebay.de/sch/i.html?_nkw=532187256</t>
         </is>
@@ -597,14 +625,20 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="G5" t="inlineStr">
+        <v>4.99</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>ExampleSeller</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>https://www.ebay.de/sch/i.html?_nkw=GX160-AF</t>
         </is>
@@ -635,14 +669,20 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="G6" t="inlineStr">
+        <v>4.99</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>ExampleSeller</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>https://www.ebay.de/sch/i.html?_nkw=P-0010038-X1HO0007</t>
         </is>

</xml_diff>

<commit_message>
refactor: map ebay api items to competitor products
</commit_message>
<xml_diff>
--- a/data/results.xlsx
+++ b/data/results.xlsx
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>4.99</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -537,13 +537,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.99</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -581,13 +581,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4.99</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4.99</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -669,13 +669,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4.99</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>

</xml_diff>